<commit_message>
Switch File 2's region filter from nationality to league played in
The Baltics/Scandinavia/Poland/Slovenia workbook was filtering by
passport country, same as the CZ/SK file. Change it to filter by which
domestic league (Wyscout file) the player actually appears in instead,
so it now picks up any nationality playing in those leagues rather than
only nationals of those countries wherever they play. CZ/SK file is
unchanged (still nationality-based, as intended).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wzh48iso9dywMF7h3c4ehR
</commit_message>
<xml_diff>
--- a/data/CZ_SK_U23_Six_Eight.xlsx
+++ b/data/CZ_SK_U23_Six_Eight.xlsx
@@ -497,7 +497,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic + Slovakia  ·  59 candidates  ·  Progressive passing + defensive-actions volume  ·  Ranked by Six Score</t>
+          <t>Czech Republic + Slovakia (by nationality)  ·  59 candidates  ·  Progressive passing + defensive-actions volume  ·  Ranked by Six Score</t>
         </is>
       </c>
     </row>
@@ -4116,7 +4116,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Czech Republic + Slovakia  ·  103 candidates  ·  Progressive passing, key passes, through passes, shot output  ·  Ranked by Eight Score</t>
+          <t>Czech Republic + Slovakia (by nationality)  ·  103 candidates  ·  Progressive passing, key passes, through passes, shot output  ·  Ranked by Eight Score</t>
         </is>
       </c>
     </row>

</xml_diff>